<commit_message>
Restore .gitignore and clean workspace
</commit_message>
<xml_diff>
--- a/ProjectMarsAutomationAdvanceTask/AdvanceTaskMars_ManulTestCases.xlsx
+++ b/ProjectMarsAutomationAdvanceTask/AdvanceTaskMars_ManulTestCases.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e476e5faad0bf1f6/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e476e5faad0bf1f6/Desktop/MarsAdvanceTask/ProjectMarsAutomationAdvanceTask/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="175" documentId="13_ncr:1_{AD277629-79CC-4ABC-BA7A-16B9D5EC8E7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{15272B94-CD07-48EB-BAE7-8497071FA7A0}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{E914B2FD-EF0C-425E-8EE6-EC6D897A5571}"/>
+    <workbookView minimized="1" xWindow="4320" yWindow="3360" windowWidth="17280" windowHeight="8880" activeTab="5" xr2:uid="{E914B2FD-EF0C-425E-8EE6-EC6D897A5571}"/>
   </bookViews>
   <sheets>
     <sheet name="Profile" sheetId="1" r:id="rId1"/>
@@ -2194,6 +2194,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2206,13 +2213,6 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2654,17 +2654,17 @@
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="B10" s="21"/>
-      <c r="C10" s="21"/>
-      <c r="D10" s="21"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="21"/>
-      <c r="G10" s="21"/>
-      <c r="H10" s="21"/>
-      <c r="I10" s="22"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="24"/>
+      <c r="I10" s="25"/>
     </row>
     <row r="11" spans="1:9" ht="76.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
@@ -2806,17 +2806,17 @@
       <c r="I15" s="1"/>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A16" s="21" t="s">
+      <c r="A16" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="B16" s="21"/>
-      <c r="C16" s="21"/>
-      <c r="D16" s="21"/>
-      <c r="E16" s="21"/>
-      <c r="F16" s="21"/>
-      <c r="G16" s="21"/>
-      <c r="H16" s="21"/>
-      <c r="I16" s="22"/>
+      <c r="B16" s="24"/>
+      <c r="C16" s="24"/>
+      <c r="D16" s="24"/>
+      <c r="E16" s="24"/>
+      <c r="F16" s="24"/>
+      <c r="G16" s="24"/>
+      <c r="H16" s="24"/>
+      <c r="I16" s="25"/>
     </row>
     <row r="17" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
@@ -2900,17 +2900,17 @@
       <c r="I19" s="1"/>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A20" s="21" t="s">
+      <c r="A20" s="24" t="s">
         <v>72</v>
       </c>
-      <c r="B20" s="21"/>
-      <c r="C20" s="21"/>
-      <c r="D20" s="21"/>
-      <c r="E20" s="21"/>
-      <c r="F20" s="21"/>
-      <c r="G20" s="21"/>
-      <c r="H20" s="21"/>
-      <c r="I20" s="22"/>
+      <c r="B20" s="24"/>
+      <c r="C20" s="24"/>
+      <c r="D20" s="24"/>
+      <c r="E20" s="24"/>
+      <c r="F20" s="24"/>
+      <c r="G20" s="24"/>
+      <c r="H20" s="24"/>
+      <c r="I20" s="25"/>
     </row>
     <row r="21" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
@@ -2969,17 +2969,17 @@
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A23" s="21" t="s">
+      <c r="A23" s="24" t="s">
         <v>79</v>
       </c>
-      <c r="B23" s="21"/>
-      <c r="C23" s="21"/>
-      <c r="D23" s="21"/>
-      <c r="E23" s="21"/>
-      <c r="F23" s="21"/>
-      <c r="G23" s="21"/>
-      <c r="H23" s="21"/>
-      <c r="I23" s="22"/>
+      <c r="B23" s="24"/>
+      <c r="C23" s="24"/>
+      <c r="D23" s="24"/>
+      <c r="E23" s="24"/>
+      <c r="F23" s="24"/>
+      <c r="G23" s="24"/>
+      <c r="H23" s="24"/>
+      <c r="I23" s="25"/>
     </row>
     <row r="24" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
@@ -3176,17 +3176,17 @@
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="B10" s="21"/>
-      <c r="C10" s="21"/>
-      <c r="D10" s="21"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="21"/>
-      <c r="G10" s="21"/>
-      <c r="H10" s="21"/>
-      <c r="I10" s="22"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="24"/>
+      <c r="I10" s="25"/>
     </row>
     <row r="11" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
@@ -3270,17 +3270,17 @@
       <c r="I13" s="1"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A14" s="21" t="s">
+      <c r="A14" s="24" t="s">
         <v>193</v>
       </c>
-      <c r="B14" s="21"/>
-      <c r="C14" s="21"/>
-      <c r="D14" s="21"/>
-      <c r="E14" s="21"/>
-      <c r="F14" s="21"/>
-      <c r="G14" s="21"/>
-      <c r="H14" s="21"/>
-      <c r="I14" s="22"/>
+      <c r="B14" s="24"/>
+      <c r="C14" s="24"/>
+      <c r="D14" s="24"/>
+      <c r="E14" s="24"/>
+      <c r="F14" s="24"/>
+      <c r="G14" s="24"/>
+      <c r="H14" s="24"/>
+      <c r="I14" s="25"/>
     </row>
     <row r="15" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
@@ -3337,17 +3337,17 @@
       <c r="I16" s="1"/>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A17" s="21" t="s">
+      <c r="A17" s="24" t="s">
         <v>194</v>
       </c>
-      <c r="B17" s="21"/>
-      <c r="C17" s="21"/>
-      <c r="D17" s="21"/>
-      <c r="E17" s="21"/>
-      <c r="F17" s="21"/>
-      <c r="G17" s="21"/>
-      <c r="H17" s="21"/>
-      <c r="I17" s="22"/>
+      <c r="B17" s="24"/>
+      <c r="C17" s="24"/>
+      <c r="D17" s="24"/>
+      <c r="E17" s="24"/>
+      <c r="F17" s="24"/>
+      <c r="G17" s="24"/>
+      <c r="H17" s="24"/>
+      <c r="I17" s="25"/>
     </row>
     <row r="18" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
@@ -3431,17 +3431,17 @@
       <c r="I20" s="1"/>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A21" s="21" t="s">
+      <c r="A21" s="24" t="s">
         <v>203</v>
       </c>
-      <c r="B21" s="21"/>
-      <c r="C21" s="21"/>
-      <c r="D21" s="21"/>
-      <c r="E21" s="21"/>
-      <c r="F21" s="21"/>
-      <c r="G21" s="21"/>
-      <c r="H21" s="21"/>
-      <c r="I21" s="22"/>
+      <c r="B21" s="24"/>
+      <c r="C21" s="24"/>
+      <c r="D21" s="24"/>
+      <c r="E21" s="24"/>
+      <c r="F21" s="24"/>
+      <c r="G21" s="24"/>
+      <c r="H21" s="24"/>
+      <c r="I21" s="25"/>
     </row>
     <row r="22" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
@@ -3552,17 +3552,17 @@
       <c r="I25" s="1"/>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A26" s="21" t="s">
+      <c r="A26" s="24" t="s">
         <v>256</v>
       </c>
-      <c r="B26" s="21"/>
-      <c r="C26" s="21"/>
-      <c r="D26" s="21"/>
-      <c r="E26" s="21"/>
-      <c r="F26" s="21"/>
-      <c r="G26" s="21"/>
-      <c r="H26" s="21"/>
-      <c r="I26" s="22"/>
+      <c r="B26" s="24"/>
+      <c r="C26" s="24"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="24"/>
+      <c r="F26" s="24"/>
+      <c r="G26" s="24"/>
+      <c r="H26" s="24"/>
+      <c r="I26" s="25"/>
     </row>
     <row r="27" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
@@ -3673,17 +3673,17 @@
       <c r="I30" s="1"/>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A31" s="21" t="s">
+      <c r="A31" s="24" t="s">
         <v>254</v>
       </c>
-      <c r="B31" s="21"/>
-      <c r="C31" s="21"/>
-      <c r="D31" s="21"/>
-      <c r="E31" s="21"/>
-      <c r="F31" s="21"/>
-      <c r="G31" s="21"/>
-      <c r="H31" s="21"/>
-      <c r="I31" s="22"/>
+      <c r="B31" s="24"/>
+      <c r="C31" s="24"/>
+      <c r="D31" s="24"/>
+      <c r="E31" s="24"/>
+      <c r="F31" s="24"/>
+      <c r="G31" s="24"/>
+      <c r="H31" s="24"/>
+      <c r="I31" s="25"/>
     </row>
     <row r="32" spans="1:9" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
@@ -3767,17 +3767,17 @@
       <c r="I34" s="1"/>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A35" s="21" t="s">
+      <c r="A35" s="24" t="s">
         <v>255</v>
       </c>
-      <c r="B35" s="21"/>
-      <c r="C35" s="21"/>
-      <c r="D35" s="21"/>
-      <c r="E35" s="21"/>
-      <c r="F35" s="21"/>
-      <c r="G35" s="21"/>
-      <c r="H35" s="21"/>
-      <c r="I35" s="22"/>
+      <c r="B35" s="24"/>
+      <c r="C35" s="24"/>
+      <c r="D35" s="24"/>
+      <c r="E35" s="24"/>
+      <c r="F35" s="24"/>
+      <c r="G35" s="24"/>
+      <c r="H35" s="24"/>
+      <c r="I35" s="25"/>
     </row>
     <row r="36" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
@@ -3861,17 +3861,17 @@
       <c r="I38" s="1"/>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A39" s="21" t="s">
+      <c r="A39" s="24" t="s">
         <v>253</v>
       </c>
-      <c r="B39" s="21"/>
-      <c r="C39" s="21"/>
-      <c r="D39" s="21"/>
-      <c r="E39" s="21"/>
-      <c r="F39" s="21"/>
-      <c r="G39" s="21"/>
-      <c r="H39" s="21"/>
-      <c r="I39" s="22"/>
+      <c r="B39" s="24"/>
+      <c r="C39" s="24"/>
+      <c r="D39" s="24"/>
+      <c r="E39" s="24"/>
+      <c r="F39" s="24"/>
+      <c r="G39" s="24"/>
+      <c r="H39" s="24"/>
+      <c r="I39" s="25"/>
     </row>
     <row r="40" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
@@ -3955,17 +3955,17 @@
       <c r="I42" s="1"/>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A43" s="21" t="s">
+      <c r="A43" s="24" t="s">
         <v>252</v>
       </c>
-      <c r="B43" s="21"/>
-      <c r="C43" s="21"/>
-      <c r="D43" s="21"/>
-      <c r="E43" s="21"/>
-      <c r="F43" s="21"/>
-      <c r="G43" s="21"/>
-      <c r="H43" s="21"/>
-      <c r="I43" s="22"/>
+      <c r="B43" s="24"/>
+      <c r="C43" s="24"/>
+      <c r="D43" s="24"/>
+      <c r="E43" s="24"/>
+      <c r="F43" s="24"/>
+      <c r="G43" s="24"/>
+      <c r="H43" s="24"/>
+      <c r="I43" s="25"/>
     </row>
     <row r="44" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
@@ -4076,17 +4076,17 @@
       <c r="I47" s="1"/>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A48" s="21" t="s">
+      <c r="A48" s="24" t="s">
         <v>251</v>
       </c>
-      <c r="B48" s="21"/>
-      <c r="C48" s="21"/>
-      <c r="D48" s="21"/>
-      <c r="E48" s="21"/>
-      <c r="F48" s="21"/>
-      <c r="G48" s="21"/>
-      <c r="H48" s="21"/>
-      <c r="I48" s="22"/>
+      <c r="B48" s="24"/>
+      <c r="C48" s="24"/>
+      <c r="D48" s="24"/>
+      <c r="E48" s="24"/>
+      <c r="F48" s="24"/>
+      <c r="G48" s="24"/>
+      <c r="H48" s="24"/>
+      <c r="I48" s="25"/>
     </row>
     <row r="49" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
@@ -4314,17 +4314,17 @@
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="B10" s="21"/>
-      <c r="C10" s="21"/>
-      <c r="D10" s="21"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="21"/>
-      <c r="G10" s="21"/>
-      <c r="H10" s="21"/>
-      <c r="I10" s="22"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="24"/>
+      <c r="I10" s="25"/>
     </row>
     <row r="11" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
@@ -4408,17 +4408,17 @@
       <c r="I13" s="1"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A14" s="21" t="s">
+      <c r="A14" s="24" t="s">
         <v>269</v>
       </c>
-      <c r="B14" s="21"/>
-      <c r="C14" s="21"/>
-      <c r="D14" s="21"/>
-      <c r="E14" s="21"/>
-      <c r="F14" s="21"/>
-      <c r="G14" s="21"/>
-      <c r="H14" s="21"/>
-      <c r="I14" s="22"/>
+      <c r="B14" s="24"/>
+      <c r="C14" s="24"/>
+      <c r="D14" s="24"/>
+      <c r="E14" s="24"/>
+      <c r="F14" s="24"/>
+      <c r="G14" s="24"/>
+      <c r="H14" s="24"/>
+      <c r="I14" s="25"/>
     </row>
     <row r="15" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
@@ -4502,17 +4502,17 @@
       <c r="I17" s="1"/>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A18" s="21" t="s">
+      <c r="A18" s="24" t="s">
         <v>272</v>
       </c>
-      <c r="B18" s="21"/>
-      <c r="C18" s="21"/>
-      <c r="D18" s="21"/>
-      <c r="E18" s="21"/>
-      <c r="F18" s="21"/>
-      <c r="G18" s="21"/>
-      <c r="H18" s="21"/>
-      <c r="I18" s="22"/>
+      <c r="B18" s="24"/>
+      <c r="C18" s="24"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="24"/>
+      <c r="F18" s="24"/>
+      <c r="G18" s="24"/>
+      <c r="H18" s="24"/>
+      <c r="I18" s="25"/>
     </row>
     <row r="19" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
@@ -4596,17 +4596,17 @@
       <c r="I21" s="1"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A22" s="21" t="s">
+      <c r="A22" s="24" t="s">
         <v>281</v>
       </c>
-      <c r="B22" s="21"/>
-      <c r="C22" s="21"/>
-      <c r="D22" s="21"/>
-      <c r="E22" s="21"/>
-      <c r="F22" s="21"/>
-      <c r="G22" s="21"/>
-      <c r="H22" s="21"/>
-      <c r="I22" s="22"/>
+      <c r="B22" s="24"/>
+      <c r="C22" s="24"/>
+      <c r="D22" s="24"/>
+      <c r="E22" s="24"/>
+      <c r="F22" s="24"/>
+      <c r="G22" s="24"/>
+      <c r="H22" s="24"/>
+      <c r="I22" s="25"/>
     </row>
     <row r="23" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
@@ -4717,17 +4717,17 @@
       <c r="I26" s="1"/>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A27" s="21" t="s">
+      <c r="A27" s="24" t="s">
         <v>289</v>
       </c>
-      <c r="B27" s="21"/>
-      <c r="C27" s="21"/>
-      <c r="D27" s="21"/>
-      <c r="E27" s="21"/>
-      <c r="F27" s="21"/>
-      <c r="G27" s="21"/>
-      <c r="H27" s="21"/>
-      <c r="I27" s="22"/>
+      <c r="B27" s="24"/>
+      <c r="C27" s="24"/>
+      <c r="D27" s="24"/>
+      <c r="E27" s="24"/>
+      <c r="F27" s="24"/>
+      <c r="G27" s="24"/>
+      <c r="H27" s="24"/>
+      <c r="I27" s="25"/>
     </row>
     <row r="28" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
@@ -4838,17 +4838,17 @@
       <c r="I31" s="1"/>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A32" s="21" t="s">
+      <c r="A32" s="24" t="s">
         <v>296</v>
       </c>
-      <c r="B32" s="21"/>
-      <c r="C32" s="21"/>
-      <c r="D32" s="21"/>
-      <c r="E32" s="21"/>
-      <c r="F32" s="21"/>
-      <c r="G32" s="21"/>
-      <c r="H32" s="21"/>
-      <c r="I32" s="22"/>
+      <c r="B32" s="24"/>
+      <c r="C32" s="24"/>
+      <c r="D32" s="24"/>
+      <c r="E32" s="24"/>
+      <c r="F32" s="24"/>
+      <c r="G32" s="24"/>
+      <c r="H32" s="24"/>
+      <c r="I32" s="25"/>
     </row>
     <row r="33" spans="1:9" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
@@ -4932,17 +4932,17 @@
       <c r="I35" s="1"/>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A36" s="21" t="s">
+      <c r="A36" s="24" t="s">
         <v>306</v>
       </c>
-      <c r="B36" s="21"/>
-      <c r="C36" s="21"/>
-      <c r="D36" s="21"/>
-      <c r="E36" s="21"/>
-      <c r="F36" s="21"/>
-      <c r="G36" s="21"/>
-      <c r="H36" s="21"/>
-      <c r="I36" s="22"/>
+      <c r="B36" s="24"/>
+      <c r="C36" s="24"/>
+      <c r="D36" s="24"/>
+      <c r="E36" s="24"/>
+      <c r="F36" s="24"/>
+      <c r="G36" s="24"/>
+      <c r="H36" s="24"/>
+      <c r="I36" s="25"/>
     </row>
     <row r="37" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
@@ -5026,17 +5026,17 @@
       <c r="I39" s="1"/>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A40" s="21" t="s">
+      <c r="A40" s="24" t="s">
         <v>316</v>
       </c>
-      <c r="B40" s="21"/>
-      <c r="C40" s="21"/>
-      <c r="D40" s="21"/>
-      <c r="E40" s="21"/>
-      <c r="F40" s="21"/>
-      <c r="G40" s="21"/>
-      <c r="H40" s="21"/>
-      <c r="I40" s="22"/>
+      <c r="B40" s="24"/>
+      <c r="C40" s="24"/>
+      <c r="D40" s="24"/>
+      <c r="E40" s="24"/>
+      <c r="F40" s="24"/>
+      <c r="G40" s="24"/>
+      <c r="H40" s="24"/>
+      <c r="I40" s="25"/>
     </row>
     <row r="41" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
@@ -5120,17 +5120,17 @@
       <c r="I43" s="1"/>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A44" s="21" t="s">
+      <c r="A44" s="24" t="s">
         <v>322</v>
       </c>
-      <c r="B44" s="21"/>
-      <c r="C44" s="21"/>
-      <c r="D44" s="21"/>
-      <c r="E44" s="21"/>
-      <c r="F44" s="21"/>
-      <c r="G44" s="21"/>
-      <c r="H44" s="21"/>
-      <c r="I44" s="22"/>
+      <c r="B44" s="24"/>
+      <c r="C44" s="24"/>
+      <c r="D44" s="24"/>
+      <c r="E44" s="24"/>
+      <c r="F44" s="24"/>
+      <c r="G44" s="24"/>
+      <c r="H44" s="24"/>
+      <c r="I44" s="25"/>
     </row>
     <row r="45" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
@@ -5241,17 +5241,17 @@
       <c r="I48" s="1"/>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A49" s="21" t="s">
+      <c r="A49" s="24" t="s">
         <v>331</v>
       </c>
-      <c r="B49" s="21"/>
-      <c r="C49" s="21"/>
-      <c r="D49" s="21"/>
-      <c r="E49" s="21"/>
-      <c r="F49" s="21"/>
-      <c r="G49" s="21"/>
-      <c r="H49" s="21"/>
-      <c r="I49" s="22"/>
+      <c r="B49" s="24"/>
+      <c r="C49" s="24"/>
+      <c r="D49" s="24"/>
+      <c r="E49" s="24"/>
+      <c r="F49" s="24"/>
+      <c r="G49" s="24"/>
+      <c r="H49" s="24"/>
+      <c r="I49" s="25"/>
     </row>
     <row r="50" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
@@ -5479,17 +5479,17 @@
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="B10" s="21"/>
-      <c r="C10" s="21"/>
-      <c r="D10" s="21"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="21"/>
-      <c r="G10" s="21"/>
-      <c r="H10" s="21"/>
-      <c r="I10" s="22"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="24"/>
+      <c r="I10" s="25"/>
     </row>
     <row r="11" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
@@ -5706,17 +5706,17 @@
       <c r="I18" s="1"/>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A19" s="21" t="s">
+      <c r="A19" s="24" t="s">
         <v>373</v>
       </c>
-      <c r="B19" s="21"/>
-      <c r="C19" s="21"/>
-      <c r="D19" s="21"/>
-      <c r="E19" s="21"/>
-      <c r="F19" s="21"/>
-      <c r="G19" s="21"/>
-      <c r="H19" s="21"/>
-      <c r="I19" s="22"/>
+      <c r="B19" s="24"/>
+      <c r="C19" s="24"/>
+      <c r="D19" s="24"/>
+      <c r="E19" s="24"/>
+      <c r="F19" s="24"/>
+      <c r="G19" s="24"/>
+      <c r="H19" s="24"/>
+      <c r="I19" s="25"/>
     </row>
     <row r="20" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
@@ -5800,17 +5800,17 @@
       <c r="I22" s="1"/>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A23" s="21" t="s">
+      <c r="A23" s="24" t="s">
         <v>386</v>
       </c>
-      <c r="B23" s="21"/>
-      <c r="C23" s="21"/>
-      <c r="D23" s="21"/>
-      <c r="E23" s="21"/>
-      <c r="F23" s="21"/>
-      <c r="G23" s="21"/>
-      <c r="H23" s="21"/>
-      <c r="I23" s="22"/>
+      <c r="B23" s="24"/>
+      <c r="C23" s="24"/>
+      <c r="D23" s="24"/>
+      <c r="E23" s="24"/>
+      <c r="F23" s="24"/>
+      <c r="G23" s="24"/>
+      <c r="H23" s="24"/>
+      <c r="I23" s="25"/>
     </row>
     <row r="24" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
@@ -5921,17 +5921,17 @@
       <c r="I27" s="1"/>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A28" s="21" t="s">
+      <c r="A28" s="24" t="s">
         <v>409</v>
       </c>
-      <c r="B28" s="21"/>
-      <c r="C28" s="21"/>
-      <c r="D28" s="21"/>
-      <c r="E28" s="21"/>
-      <c r="F28" s="21"/>
-      <c r="G28" s="21"/>
-      <c r="H28" s="21"/>
-      <c r="I28" s="22"/>
+      <c r="B28" s="24"/>
+      <c r="C28" s="24"/>
+      <c r="D28" s="24"/>
+      <c r="E28" s="24"/>
+      <c r="F28" s="24"/>
+      <c r="G28" s="24"/>
+      <c r="H28" s="24"/>
+      <c r="I28" s="25"/>
     </row>
     <row r="29" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
@@ -6219,17 +6219,17 @@
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A13" s="21" t="s">
+      <c r="A13" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="B13" s="21"/>
-      <c r="C13" s="21"/>
-      <c r="D13" s="21"/>
-      <c r="E13" s="21"/>
-      <c r="F13" s="21"/>
-      <c r="G13" s="21"/>
-      <c r="H13" s="21"/>
-      <c r="I13" s="22"/>
+      <c r="B13" s="24"/>
+      <c r="C13" s="24"/>
+      <c r="D13" s="24"/>
+      <c r="E13" s="24"/>
+      <c r="F13" s="24"/>
+      <c r="G13" s="24"/>
+      <c r="H13" s="24"/>
+      <c r="I13" s="25"/>
     </row>
     <row r="14" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
@@ -6313,44 +6313,44 @@
       <c r="I16" s="16"/>
     </row>
     <row r="17" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="23" t="s">
+      <c r="A17" s="26" t="s">
         <v>425</v>
       </c>
-      <c r="B17" s="23" t="s">
+      <c r="B17" s="26" t="s">
         <v>426</v>
       </c>
-      <c r="C17" s="23" t="s">
+      <c r="C17" s="26" t="s">
         <v>427</v>
       </c>
       <c r="D17" s="16" t="s">
         <v>428</v>
       </c>
-      <c r="E17" s="23" t="s">
+      <c r="E17" s="26" t="s">
         <v>430</v>
       </c>
-      <c r="F17" s="23" t="s">
+      <c r="F17" s="26" t="s">
         <v>431</v>
       </c>
-      <c r="G17" s="23" t="s">
+      <c r="G17" s="26" t="s">
         <v>431</v>
       </c>
-      <c r="H17" s="24" t="s">
-        <v>26</v>
-      </c>
-      <c r="I17" s="23"/>
+      <c r="H17" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="I17" s="26"/>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A18" s="23"/>
-      <c r="B18" s="23"/>
-      <c r="C18" s="23"/>
+      <c r="A18" s="26"/>
+      <c r="B18" s="26"/>
+      <c r="C18" s="26"/>
       <c r="D18" s="16" t="s">
         <v>429</v>
       </c>
-      <c r="E18" s="23"/>
-      <c r="F18" s="23"/>
-      <c r="G18" s="23"/>
-      <c r="H18" s="24"/>
-      <c r="I18" s="23"/>
+      <c r="E18" s="26"/>
+      <c r="F18" s="26"/>
+      <c r="G18" s="26"/>
+      <c r="H18" s="27"/>
+      <c r="I18" s="26"/>
     </row>
     <row r="19" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="16" t="s">
@@ -6542,17 +6542,17 @@
       <c r="I25" s="16"/>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A26" s="21" t="s">
+      <c r="A26" s="24" t="s">
         <v>457</v>
       </c>
-      <c r="B26" s="21"/>
-      <c r="C26" s="21"/>
-      <c r="D26" s="21"/>
-      <c r="E26" s="21"/>
-      <c r="F26" s="21"/>
-      <c r="G26" s="21"/>
-      <c r="H26" s="21"/>
-      <c r="I26" s="22"/>
+      <c r="B26" s="24"/>
+      <c r="C26" s="24"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="24"/>
+      <c r="F26" s="24"/>
+      <c r="G26" s="24"/>
+      <c r="H26" s="24"/>
+      <c r="I26" s="25"/>
     </row>
     <row r="27" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A27" s="16" t="s">
@@ -6603,7 +6603,7 @@
       <c r="G28" s="16" t="s">
         <v>595</v>
       </c>
-      <c r="H28" s="25" t="s">
+      <c r="H28" s="22" t="s">
         <v>357</v>
       </c>
       <c r="I28" s="16"/>
@@ -6620,17 +6620,17 @@
       <c r="I29" s="16"/>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A30" s="21" t="s">
+      <c r="A30" s="24" t="s">
         <v>458</v>
       </c>
-      <c r="B30" s="21"/>
-      <c r="C30" s="21"/>
-      <c r="D30" s="21"/>
-      <c r="E30" s="21"/>
-      <c r="F30" s="21"/>
-      <c r="G30" s="21"/>
-      <c r="H30" s="21"/>
-      <c r="I30" s="22"/>
+      <c r="B30" s="24"/>
+      <c r="C30" s="24"/>
+      <c r="D30" s="24"/>
+      <c r="E30" s="24"/>
+      <c r="F30" s="24"/>
+      <c r="G30" s="24"/>
+      <c r="H30" s="24"/>
+      <c r="I30" s="25"/>
     </row>
     <row r="31" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A31" s="16" t="s">
@@ -6681,7 +6681,7 @@
       <c r="G32" s="1" t="s">
         <v>596</v>
       </c>
-      <c r="H32" s="25" t="s">
+      <c r="H32" s="22" t="s">
         <v>357</v>
       </c>
       <c r="I32" s="1"/>
@@ -6714,17 +6714,17 @@
       <c r="I33" s="1"/>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A34" s="21" t="s">
+      <c r="A34" s="24" t="s">
         <v>487</v>
       </c>
-      <c r="B34" s="21"/>
-      <c r="C34" s="21"/>
-      <c r="D34" s="21"/>
-      <c r="E34" s="21"/>
-      <c r="F34" s="21"/>
-      <c r="G34" s="21"/>
-      <c r="H34" s="21"/>
-      <c r="I34" s="22"/>
+      <c r="B34" s="24"/>
+      <c r="C34" s="24"/>
+      <c r="D34" s="24"/>
+      <c r="E34" s="24"/>
+      <c r="F34" s="24"/>
+      <c r="G34" s="24"/>
+      <c r="H34" s="24"/>
+      <c r="I34" s="25"/>
     </row>
     <row r="35" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A35" s="16" t="s">
@@ -7026,17 +7026,17 @@
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A13" s="21" t="s">
+      <c r="A13" s="24" t="s">
         <v>607</v>
       </c>
-      <c r="B13" s="21"/>
-      <c r="C13" s="21"/>
-      <c r="D13" s="21"/>
-      <c r="E13" s="21"/>
-      <c r="F13" s="21"/>
-      <c r="G13" s="21"/>
-      <c r="H13" s="21"/>
-      <c r="I13" s="22"/>
+      <c r="B13" s="24"/>
+      <c r="C13" s="24"/>
+      <c r="D13" s="24"/>
+      <c r="E13" s="24"/>
+      <c r="F13" s="24"/>
+      <c r="G13" s="24"/>
+      <c r="H13" s="24"/>
+      <c r="I13" s="25"/>
     </row>
     <row r="14" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A14" s="16" t="s">
@@ -7060,50 +7060,50 @@
       <c r="G14" s="16" t="s">
         <v>505</v>
       </c>
-      <c r="H14" s="26" t="s">
+      <c r="H14" s="21" t="s">
         <v>26</v>
       </c>
       <c r="I14" s="16"/>
     </row>
     <row r="15" spans="1:9" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="23" t="s">
+      <c r="A15" s="26" t="s">
         <v>506</v>
       </c>
-      <c r="B15" s="23" t="s">
+      <c r="B15" s="26" t="s">
         <v>507</v>
       </c>
-      <c r="C15" s="23" t="s">
+      <c r="C15" s="26" t="s">
         <v>508</v>
       </c>
       <c r="D15" s="16" t="s">
         <v>509</v>
       </c>
-      <c r="E15" s="23" t="s">
+      <c r="E15" s="26" t="s">
         <v>413</v>
       </c>
-      <c r="F15" s="23" t="s">
+      <c r="F15" s="26" t="s">
         <v>510</v>
       </c>
-      <c r="G15" s="23" t="s">
+      <c r="G15" s="26" t="s">
         <v>510</v>
       </c>
-      <c r="H15" s="24" t="s">
-        <v>26</v>
-      </c>
-      <c r="I15" s="23"/>
+      <c r="H15" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="I15" s="26"/>
     </row>
     <row r="16" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A16" s="23"/>
-      <c r="B16" s="23"/>
-      <c r="C16" s="23"/>
+      <c r="A16" s="26"/>
+      <c r="B16" s="26"/>
+      <c r="C16" s="26"/>
       <c r="D16" s="16" t="s">
         <v>594</v>
       </c>
-      <c r="E16" s="23"/>
-      <c r="F16" s="23"/>
-      <c r="G16" s="23"/>
-      <c r="H16" s="24"/>
-      <c r="I16" s="23"/>
+      <c r="E16" s="26"/>
+      <c r="F16" s="26"/>
+      <c r="G16" s="26"/>
+      <c r="H16" s="27"/>
+      <c r="I16" s="26"/>
     </row>
     <row r="17" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A17" s="16" t="s">
@@ -7127,7 +7127,7 @@
       <c r="G17" s="16" t="s">
         <v>515</v>
       </c>
-      <c r="H17" s="26" t="s">
+      <c r="H17" s="21" t="s">
         <v>26</v>
       </c>
       <c r="I17" s="16"/>
@@ -7154,7 +7154,7 @@
       <c r="G18" s="16" t="s">
         <v>519</v>
       </c>
-      <c r="H18" s="26" t="s">
+      <c r="H18" s="21" t="s">
         <v>26</v>
       </c>
       <c r="I18" s="16"/>
@@ -7181,7 +7181,7 @@
       <c r="G19" s="16" t="s">
         <v>524</v>
       </c>
-      <c r="H19" s="26" t="s">
+      <c r="H19" s="21" t="s">
         <v>26</v>
       </c>
       <c r="I19" s="16"/>
@@ -7208,11 +7208,11 @@
       <c r="G20" s="16" t="s">
         <v>529</v>
       </c>
-      <c r="H20" s="26" t="s">
+      <c r="H20" s="21" t="s">
         <v>26</v>
       </c>
       <c r="I20" s="16"/>
-      <c r="K20" s="27"/>
+      <c r="K20" s="23"/>
     </row>
     <row r="21" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A21" s="16" t="s">
@@ -7236,7 +7236,7 @@
       <c r="G21" s="16" t="s">
         <v>533</v>
       </c>
-      <c r="H21" s="26" t="s">
+      <c r="H21" s="21" t="s">
         <v>26</v>
       </c>
       <c r="I21" s="16"/>
@@ -7263,7 +7263,7 @@
       <c r="G22" s="16" t="s">
         <v>538</v>
       </c>
-      <c r="H22" s="26" t="s">
+      <c r="H22" s="21" t="s">
         <v>26</v>
       </c>
       <c r="I22" s="16"/>
@@ -7290,7 +7290,7 @@
       <c r="G23" s="16" t="s">
         <v>543</v>
       </c>
-      <c r="H23" s="26" t="s">
+      <c r="H23" s="21" t="s">
         <v>26</v>
       </c>
       <c r="I23" s="16"/>
@@ -7317,7 +7317,7 @@
       <c r="G24" s="16" t="s">
         <v>548</v>
       </c>
-      <c r="H24" s="26" t="s">
+      <c r="H24" s="21" t="s">
         <v>26</v>
       </c>
       <c r="I24" s="16"/>
@@ -7344,7 +7344,7 @@
       <c r="G25" s="16" t="s">
         <v>606</v>
       </c>
-      <c r="H25" s="26" t="s">
+      <c r="H25" s="21" t="s">
         <v>26</v>
       </c>
       <c r="I25" s="16"/>
@@ -7371,7 +7371,7 @@
       <c r="G26" s="16" t="s">
         <v>557</v>
       </c>
-      <c r="H26" s="26" t="s">
+      <c r="H26" s="21" t="s">
         <v>26</v>
       </c>
       <c r="I26" s="16"/>
@@ -7398,7 +7398,7 @@
       <c r="G27" s="16" t="s">
         <v>562</v>
       </c>
-      <c r="H27" s="26" t="s">
+      <c r="H27" s="21" t="s">
         <v>26</v>
       </c>
       <c r="I27" s="16"/>
@@ -7425,7 +7425,7 @@
       <c r="G28" s="16" t="s">
         <v>567</v>
       </c>
-      <c r="H28" s="26" t="s">
+      <c r="H28" s="21" t="s">
         <v>26</v>
       </c>
       <c r="I28" s="16"/>
@@ -7452,7 +7452,7 @@
       <c r="G29" s="16" t="s">
         <v>571</v>
       </c>
-      <c r="H29" s="26" t="s">
+      <c r="H29" s="21" t="s">
         <v>26</v>
       </c>
       <c r="I29" s="16"/>
@@ -7479,11 +7479,11 @@
       <c r="G30" s="16" t="s">
         <v>575</v>
       </c>
-      <c r="H30" s="26" t="s">
+      <c r="H30" s="21" t="s">
         <v>26</v>
       </c>
       <c r="I30" s="16"/>
-      <c r="J30" s="27"/>
+      <c r="J30" s="23"/>
     </row>
     <row r="31" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A31" s="16" t="s">
@@ -7507,7 +7507,7 @@
       <c r="G31" s="16" t="s">
         <v>580</v>
       </c>
-      <c r="H31" s="26" t="s">
+      <c r="H31" s="21" t="s">
         <v>26</v>
       </c>
       <c r="I31" s="16"/>
@@ -7534,7 +7534,7 @@
       <c r="G32" s="16" t="s">
         <v>585</v>
       </c>
-      <c r="H32" s="26" t="s">
+      <c r="H32" s="21" t="s">
         <v>26</v>
       </c>
       <c r="I32" s="16"/>
@@ -7561,7 +7561,7 @@
       <c r="G33" s="16" t="s">
         <v>589</v>
       </c>
-      <c r="H33" s="26" t="s">
+      <c r="H33" s="21" t="s">
         <v>26</v>
       </c>
       <c r="I33" s="16"/>
@@ -7588,7 +7588,7 @@
       <c r="G34" s="16" t="s">
         <v>593</v>
       </c>
-      <c r="H34" s="26" t="s">
+      <c r="H34" s="21" t="s">
         <v>26</v>
       </c>
       <c r="I34" s="16"/>

</xml_diff>